<commit_message>
excel_row_index = job_index + 2  # NOTE Ichanged this to +1 and it changes the ast_condition header row to Failed. So it must stay at +2
 ast_condition column seems to be fixed after some changes. Now need to work on dont_overwrite_outputs to true missing the first row.
</commit_message>
<xml_diff>
--- a/autoast/jobs_to_fail_FAST.xlsx
+++ b/autoast/jobs_to_fail_FAST.xlsx
@@ -781,7 +781,7 @@
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="I5" s="1" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>Requeued</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="N6" s="3" t="n">

</xml_diff>